<commit_message>
Add Motive integration and connection documentation
</commit_message>
<xml_diff>
--- a/vehicles.xlsx
+++ b/vehicles.xlsx
@@ -93,7 +93,7 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>OTOS</t>
+    <t>localization/odom</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -493,7 +493,7 @@
     <col min="3" max="3" width="23.75" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.625" customWidth="1"/>
     <col min="6" max="6" width="8.625" customWidth="1"/>
-    <col min="7" max="7" width="10.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.25" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>